<commit_message>
who even knows whats going on atp
</commit_message>
<xml_diff>
--- a/script1/registered_scored.xlsx
+++ b/script1/registered_scored.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -547,17 +547,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Baldwin, Dan</t>
+          <t>Abel, Caiden</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1099776</t>
+          <t>1100036</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>DWBaldwin</t>
+          <t>1182664</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -581,17 +581,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>De, Sanchari</t>
+          <t>Baxter, Jessica</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1099776</t>
+          <t>1100036</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>SDe</t>
+          <t>JABaxter</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
@@ -615,17 +615,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Fuentes, Victor</t>
+          <t>Brewer, Courtney</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1099776</t>
+          <t>1100036</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>vfuentesjr442</t>
+          <t>1180013</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -649,17 +649,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Gallardo, Juan</t>
+          <t>Brewer, Elijah</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1099776</t>
+          <t>1100036</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>JGallardo</t>
+          <t>1183489</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -683,17 +683,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Harrell, chris</t>
+          <t>Cavazos, Elyssia</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1099776</t>
+          <t>1100036</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1181212</t>
+          <t>ecavazos</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -717,17 +717,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Hearn, Jim</t>
+          <t>Deis, Sandra</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1099776</t>
+          <t>1100036</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>210438</t>
+          <t>SDeis</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -751,17 +751,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Le Morvan, Isaac</t>
+          <t>Dequillettes, Woody</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1099776</t>
+          <t>1100036</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1181899</t>
+          <t>wdequillettes</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -785,17 +785,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Lehman, Nicholas</t>
+          <t>Desabrais, Duke</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1099776</t>
+          <t>1100036</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1101620</t>
+          <t>DDDesabrais</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -809,7 +809,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
@@ -819,17 +819,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Mohammad, Ahmad</t>
+          <t>Fultz, Melissa</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1099776</t>
+          <t>1100036</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1111013</t>
+          <t>1182139</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -853,17 +853,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Patrick, Miranda</t>
+          <t>Graydon Jr., David</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1099776</t>
+          <t>1100036</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1180745</t>
+          <t>1183337</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -877,7 +877,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
@@ -887,17 +887,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Reiff, Zoe</t>
+          <t>Gross, Landon</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1099776</t>
+          <t>1100036</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1180968</t>
+          <t>LRGross</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
@@ -921,17 +921,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Singh, Corey</t>
+          <t>Haile, Kokob</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>1099776</t>
+          <t>1100036</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CASingh</t>
+          <t>1104534</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
@@ -955,17 +955,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Sofan, Mohammad</t>
+          <t>Huggins, Steve</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1099776</t>
+          <t>1100036</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>MSofan</t>
+          <t>1181516</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -979,7 +979,7 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
@@ -989,17 +989,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Thomas, Scott</t>
+          <t>Ikonomakis, George</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1099776</t>
+          <t>1100036</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1180589</t>
+          <t>196427</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1023,17 +1023,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Ziha, Jaafar</t>
+          <t>Iqbal, Aban</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1099776</t>
+          <t>1100036</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>203091</t>
+          <t>1181094</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1047,13 +1047,931 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Jabbour, Karim</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1181558</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Jatzke, Nicole</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1182885</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>K C, Himamsu</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>207477</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Kedowide, Cyrian</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1102855</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Knox, Dakota</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>1182538</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Kuysters, Jordan</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>1183254</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Mace, Maria</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>202596</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Mancini, Meagan</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>MMancini</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Massie, Dillon</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>1180982</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Maxfield, Alisha</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>1181978</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>McIvor, Bailey</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1182701</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Mestdagh, Karlee</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>1103306</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Molinski, Vanessa</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>204560</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Nasrallah, Anthony</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>1182739</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>O'Brien, Amy</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1182666</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Opdendries, Mike</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>MOpdendries</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Percy, Taylor</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>1182766</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Profiri, Ben</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>1183553</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Schieber, Adam</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>1114738</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Seelig, Bella</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>1182770</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Sharifi, Sherry</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>205653</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Smith, Beth</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>1181616</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Tadesse, Elim</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>1183461</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Ushkowski, Logan</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>1183136</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Velez, Javier</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>1181908</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Williams, Ashley</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>1182639</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Zubko, Kenzie</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1100036</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>1181973</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>